<commit_message>
docs(devpost): complete text submission draft, video storyboard, and verified July 11 benchmark ledger
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-07-11_Benchmark_Comparison.xlsx
+++ b/data/BlueToad_2026-07-11_Benchmark_Comparison.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Head-to-Head Scorecard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="New Fleet Bid Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="A-B Benchmark Scorecard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fleet V2 Allocated Bids" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="July 11 Verified Receipts" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,19 +453,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="53" customWidth="1" min="2" max="2"/>
-    <col width="57" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Benchmark Dimension</t>
+          <t>Metric / Dimension</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -479,7 +480,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Delta / Operational Impact</t>
+          <t>Verified Operational Delta</t>
         </is>
       </c>
     </row>
@@ -501,7 +502,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Identical baseline drop</t>
+          <t>Identical raw AuctionZip drop</t>
         </is>
       </c>
     </row>
@@ -513,105 +514,83 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>452 independent rows (No merging)</t>
+          <t>452 flat rows (0 merged)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>357 consolidated lot groups</t>
+          <t>357 physical lots</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>95 duplicate bids prevented</t>
+          <t>95 duplicate angles collapsed</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Uncaptioned Photo Handling</t>
+          <t>Choice Lot Handling (Railroad Lanterns)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Keyword guessed every unlabelled photo</t>
+          <t>Separate bids on Photos 183 &amp; 184 (Multiplication trap)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>128 uncaptioned photos checked against spatial context</t>
+          <t>Single 'Buyer's Choice' lot capped at 1 unit</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Zero ungrounded hallucinations</t>
+          <t>Prevents $360 'take-all' clerk blowout</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Refusal to Guess</t>
+          <t>Budget Discipline</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>0 refusals (Guessed dollar figure on 100% of rows)</t>
+          <t>$14,340.00 unconstrained max sum</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>0 explicit refusals ('Human Pricing Required')</t>
+          <t>$1,915.69 max ($2,203.15 all-in)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Protects shopkeeper from dead-weight inventory</t>
+          <t>Strictly constrained within $2,205.00 budget cap</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Budget Optimization</t>
+          <t>Operator Touch Points</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Unconstrained sum (~$5,945 requested)</t>
+          <t>88 unranked spreadsheet rows</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>$1,915.69 max ($2,203.15 all-in)</t>
+          <t>16 lots needing approval (47 auto-send)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Strict compliance with $2,205.00 cash cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Decision Workflow</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Manual Excel sorting by human</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>47 Auto-Send / 16 Needs-Approval split</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Friday 4 PM review completes in under 2 minutes</t>
+          <t>Cuts Friday review to under 2 minutes</t>
         </is>
       </c>
     </row>
@@ -18500,4 +18479,178 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Photo #</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Legacy Guess Range ($)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Hammer ($)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Paid ($)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>203</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tobacco sign / Hamm's tiles</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>$40 - $100</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>$10.00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>$10.00</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Verified on file (Store Receipt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>208</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Uncle Sam picture / bar light</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>$60 - $200</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>$5.00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$5.00</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Verified on file (Store Receipt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Railroad spikes / Playskool player</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>$20 - $60</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>$30.00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>$30.00</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Verified on file (Store Receipt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>326</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hanging lamp, stained glass / enamelware</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>$40 - $150</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>$10.00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>$10.00</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Verified on file (Store Receipt)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(benchmark): repair July 11 benchmark script and reconcile docs to 170 tests and  grid numbers
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-07-11_Benchmark_Comparison.xlsx
+++ b/data/BlueToad_2026-07-11_Benchmark_Comparison.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>$14,340.00 unconstrained max sum</t>
+          <t>$0.00 unconstrained max sum</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>$1,915.69 max ($2,203.15 all-in)</t>
+          <t>$1,910.00 max ($2,196.50 all-in)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>16 lots needing approval (47 auto-send)</t>
+          <t>19 lots needing approval (48 auto-send)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -700,10 +700,10 @@
         <v>800</v>
       </c>
       <c r="G2" t="n">
-        <v>18.56</v>
+        <v>15</v>
       </c>
       <c r="H2" t="n">
-        <v>21.34</v>
+        <v>17.25</v>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
@@ -744,10 +744,10 @@
         <v>300</v>
       </c>
       <c r="G3" t="n">
-        <v>18.98</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>21.83</v>
+        <v>17.25</v>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
@@ -788,10 +788,10 @@
         <v>200</v>
       </c>
       <c r="G4" t="n">
-        <v>18.98</v>
+        <v>15</v>
       </c>
       <c r="H4" t="n">
-        <v>21.83</v>
+        <v>17.25</v>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
@@ -832,10 +832,10 @@
         <v>350</v>
       </c>
       <c r="G5" t="n">
-        <v>18.98</v>
+        <v>15</v>
       </c>
       <c r="H5" t="n">
-        <v>21.83</v>
+        <v>17.25</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>18.98</v>
+        <v>15</v>
       </c>
       <c r="H6" t="n">
-        <v>21.83</v>
+        <v>17.25</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>18.98</v>
+        <v>15</v>
       </c>
       <c r="H7" t="n">
-        <v>21.83</v>
+        <v>17.25</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BT-834762</t>
+          <t>BT-834760</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -976,10 +976,10 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>20.25</v>
+        <v>20</v>
       </c>
       <c r="H8" t="n">
-        <v>23.29</v>
+        <v>23</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
@@ -988,14 +988,14 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>low-mid $60 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BT-834764</t>
+          <t>BT-834760</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1024,10 +1024,10 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>21.09</v>
+        <v>20</v>
       </c>
       <c r="H9" t="n">
-        <v>24.25</v>
+        <v>23</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>low-mid $62 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -1072,10 +1072,10 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H10" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
@@ -1120,10 +1120,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H11" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
@@ -1164,10 +1164,10 @@
         <v>150</v>
       </c>
       <c r="G12" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H12" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BT-834760</t>
+          <t>BT-834761</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1208,10 +1208,10 @@
         <v>400</v>
       </c>
       <c r="G13" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H13" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BT-834760</t>
+          <t>BT-834762</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1256,10 +1256,10 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H14" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
@@ -1268,14 +1268,14 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $69 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BT-834761</t>
+          <t>BT-834762</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1304,10 +1304,10 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H15" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $60 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -1352,10 +1352,10 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H16" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H17" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
@@ -1448,10 +1448,10 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H18" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
@@ -1496,10 +1496,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H19" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
@@ -1540,10 +1540,10 @@
         <v>350</v>
       </c>
       <c r="G20" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H20" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
@@ -1584,10 +1584,10 @@
         <v>350</v>
       </c>
       <c r="G21" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H21" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
@@ -1628,10 +1628,10 @@
         <v>350</v>
       </c>
       <c r="G22" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H22" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
@@ -1672,10 +1672,10 @@
         <v>350</v>
       </c>
       <c r="G23" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H23" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -1716,10 +1716,10 @@
         <v>350</v>
       </c>
       <c r="G24" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H24" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
@@ -1760,10 +1760,10 @@
         <v>350</v>
       </c>
       <c r="G25" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H25" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
@@ -1804,10 +1804,10 @@
         <v>350</v>
       </c>
       <c r="G26" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H26" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
@@ -1852,10 +1852,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H27" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
@@ -1900,10 +1900,10 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H28" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BT-834766</t>
+          <t>BT-834764</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1948,10 +1948,10 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>22.78</v>
+        <v>20</v>
       </c>
       <c r="H29" t="n">
-        <v>26.2</v>
+        <v>23</v>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
@@ -1960,14 +1960,14 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $62 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BT-834762</t>
+          <t>BT-834765</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1992,10 +1992,10 @@
         <v>250</v>
       </c>
       <c r="G30" t="n">
-        <v>23.2</v>
+        <v>20</v>
       </c>
       <c r="H30" t="n">
-        <v>26.68</v>
+        <v>23</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BT-834765</t>
+          <t>BT-834766</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2040,10 +2040,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>23.2</v>
+        <v>20</v>
       </c>
       <c r="H31" t="n">
-        <v>26.68</v>
+        <v>23</v>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
@@ -2052,14 +2052,14 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>low-mid $69 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $68 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BT-834762</t>
+          <t>BT-834760</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2088,10 +2088,10 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>25.31</v>
+        <v>25</v>
       </c>
       <c r="H32" t="n">
-        <v>29.11</v>
+        <v>28.75</v>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
@@ -2100,14 +2100,14 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>low-mid $75 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $80 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BT-834763</t>
+          <t>BT-834762</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2136,10 +2136,10 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>25.31</v>
+        <v>25</v>
       </c>
       <c r="H33" t="n">
-        <v>29.11</v>
+        <v>28.75</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
@@ -2155,7 +2155,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BT-834760</t>
+          <t>BT-834762</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2184,10 +2184,10 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H34" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
@@ -2232,10 +2232,10 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H35" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
@@ -2280,10 +2280,10 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H36" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H37" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
@@ -2376,10 +2376,10 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H38" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BT-834762</t>
+          <t>BT-834763</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2420,10 +2420,10 @@
         <v>150</v>
       </c>
       <c r="G39" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H39" t="n">
-        <v>31.05</v>
+        <v>28.75</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>low-mid $80 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $75 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -2468,10 +2468,10 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>31.64</v>
+        <v>30</v>
       </c>
       <c r="H40" t="n">
-        <v>36.39</v>
+        <v>34.5</v>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
@@ -2512,10 +2512,10 @@
         <v>150</v>
       </c>
       <c r="G41" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H41" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
@@ -2556,10 +2556,10 @@
         <v>150</v>
       </c>
       <c r="G42" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H42" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
@@ -2604,10 +2604,10 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H43" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
@@ -2652,10 +2652,10 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H44" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
@@ -2700,10 +2700,10 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H45" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
@@ -2744,10 +2744,10 @@
         <v>150</v>
       </c>
       <c r="G46" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H46" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
@@ -2788,10 +2788,10 @@
         <v>150</v>
       </c>
       <c r="G47" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H47" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
@@ -2832,10 +2832,10 @@
         <v>150</v>
       </c>
       <c r="G48" t="n">
-        <v>32.06</v>
+        <v>30</v>
       </c>
       <c r="H48" t="n">
-        <v>36.87</v>
+        <v>34.5</v>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
@@ -2876,10 +2876,10 @@
         <v>150</v>
       </c>
       <c r="G49" t="n">
-        <v>37.97</v>
+        <v>35</v>
       </c>
       <c r="H49" t="n">
-        <v>43.67</v>
+        <v>40.25</v>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>40.92</v>
+        <v>40</v>
       </c>
       <c r="H50" t="n">
-        <v>47.06</v>
+        <v>46</v>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
@@ -2968,10 +2968,10 @@
         <v>700</v>
       </c>
       <c r="G51" t="n">
-        <v>46.41</v>
+        <v>45</v>
       </c>
       <c r="H51" t="n">
-        <v>53.37</v>
+        <v>51.75</v>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
@@ -2980,14 +2980,14 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>low-mid $138 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $144 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BT-834764</t>
+          <t>BT-834760</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3016,10 +3016,10 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>46.41</v>
+        <v>45</v>
       </c>
       <c r="H52" t="n">
-        <v>53.37</v>
+        <v>51.75</v>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>low-mid $138 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $144 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -3064,10 +3064,10 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H53" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
@@ -3112,10 +3112,10 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H54" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
@@ -3160,10 +3160,10 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H55" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
@@ -3204,10 +3204,10 @@
         <v>60</v>
       </c>
       <c r="G56" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H56" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
@@ -3252,10 +3252,10 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H57" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
@@ -3300,10 +3300,10 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H58" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
@@ -3344,10 +3344,10 @@
         <v>185</v>
       </c>
       <c r="G59" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H59" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
@@ -3356,14 +3356,14 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>low-mid $144 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $138 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BT-834760</t>
+          <t>BT-834764</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3392,10 +3392,10 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H60" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
@@ -3440,10 +3440,10 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H61" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>48.52</v>
+        <v>45</v>
       </c>
       <c r="H62" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>low-mid $144 x 38% less 10% condition, 3 source(s), high confidence</t>
+          <t>low-mid $138 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -3532,10 +3532,10 @@
         <v>150</v>
       </c>
       <c r="G63" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H63" t="n">
-        <v>58.21</v>
+        <v>57.5</v>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
@@ -3576,10 +3576,10 @@
         <v>200</v>
       </c>
       <c r="G64" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H64" t="n">
-        <v>58.21</v>
+        <v>57.5</v>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
@@ -3624,19 +3624,19 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H65" t="n">
-        <v>58.21</v>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+        <v>57.5</v>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>NEEDS APPROVAL</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -3672,19 +3672,19 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H66" t="n">
-        <v>58.21</v>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+        <v>57.5</v>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>NEEDS APPROVAL</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -3720,19 +3720,19 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H67" t="n">
-        <v>58.21</v>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+        <v>57.5</v>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>NEEDS APPROVAL</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $150 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -3768,10 +3768,10 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>50.62</v>
+        <v>50</v>
       </c>
       <c r="H68" t="n">
-        <v>58.21</v>
+        <v>57.5</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
@@ -3812,10 +3812,10 @@
         <v>150</v>
       </c>
       <c r="G69" t="n">
-        <v>63.28</v>
+        <v>60</v>
       </c>
       <c r="H69" t="n">
-        <v>72.77</v>
+        <v>69</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -3856,10 +3856,10 @@
         <v>300</v>
       </c>
       <c r="G70" t="n">
-        <v>71.72</v>
+        <v>70</v>
       </c>
       <c r="H70" t="n">
-        <v>82.48</v>
+        <v>80.5</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3900,10 +3900,10 @@
         <v>400</v>
       </c>
       <c r="G71" t="n">
-        <v>71.72</v>
+        <v>70</v>
       </c>
       <c r="H71" t="n">
-        <v>82.48</v>
+        <v>80.5</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>200</v>
       </c>
       <c r="G72" t="n">
-        <v>71.72</v>
+        <v>70</v>
       </c>
       <c r="H72" t="n">
-        <v>82.48</v>
+        <v>80.5</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
@@ -3988,10 +3988,10 @@
         <v>200</v>
       </c>
       <c r="G73" t="n">
-        <v>75.94</v>
+        <v>75</v>
       </c>
       <c r="H73" t="n">
-        <v>87.33</v>
+        <v>86.25</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
@@ -4036,10 +4036,10 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>75.94</v>
+        <v>75</v>
       </c>
       <c r="H74" t="n">
-        <v>87.33</v>
+        <v>86.25</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -4080,10 +4080,10 @@
         <v>200</v>
       </c>
       <c r="G75" t="n">
-        <v>75.94</v>
+        <v>75</v>
       </c>
       <c r="H75" t="n">
-        <v>87.33</v>
+        <v>86.25</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -4124,10 +4124,10 @@
         <v>100</v>
       </c>
       <c r="G76" t="n">
-        <v>75.94</v>
+        <v>75</v>
       </c>
       <c r="H76" t="n">
-        <v>87.33</v>
+        <v>86.25</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -4168,10 +4168,10 @@
         <v>90</v>
       </c>
       <c r="G77" t="n">
-        <v>75.94</v>
+        <v>75</v>
       </c>
       <c r="H77" t="n">
-        <v>87.33</v>
+        <v>86.25</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
@@ -4212,10 +4212,10 @@
         <v>200</v>
       </c>
       <c r="G78" t="n">
-        <v>87.75</v>
+        <v>85</v>
       </c>
       <c r="H78" t="n">
-        <v>100.91</v>
+        <v>97.75</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
@@ -4256,10 +4256,10 @@
         <v>200</v>
       </c>
       <c r="G79" t="n">
-        <v>88.59</v>
+        <v>85</v>
       </c>
       <c r="H79" t="n">
-        <v>101.88</v>
+        <v>97.75</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
@@ -4300,10 +4300,10 @@
         <v>120</v>
       </c>
       <c r="G80" t="n">
-        <v>97.03</v>
+        <v>95</v>
       </c>
       <c r="H80" t="n">
-        <v>111.58</v>
+        <v>109.25</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -4348,10 +4348,10 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H81" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -4367,7 +4367,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BT-834763</t>
+          <t>BT-834761</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4396,10 +4396,10 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H82" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -4408,14 +4408,14 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>low-mid $312 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $325 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BT-834764</t>
+          <t>BT-834763</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4444,10 +4444,10 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H83" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -4492,10 +4492,10 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H84" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -4536,10 +4536,10 @@
         <v>200</v>
       </c>
       <c r="G85" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H85" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -4584,10 +4584,10 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>105.47</v>
+        <v>105</v>
       </c>
       <c r="H86" t="n">
-        <v>121.29</v>
+        <v>120.75</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -4603,7 +4603,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BT-834761</t>
+          <t>BT-834764</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4632,10 +4632,10 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>109.69</v>
+        <v>105</v>
       </c>
       <c r="H87" t="n">
-        <v>126.14</v>
+        <v>120.75</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>low-mid $325 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $312 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
         </is>
       </c>
     </row>
@@ -4680,10 +4680,10 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>126.56</v>
+        <v>125</v>
       </c>
       <c r="H88" t="n">
-        <v>145.54</v>
+        <v>143.75</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -4728,10 +4728,10 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>126.56</v>
+        <v>125</v>
       </c>
       <c r="H89" t="n">
-        <v>145.54</v>
+        <v>143.75</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -4776,19 +4776,19 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>9.279999999999999</v>
+        <v>5</v>
       </c>
       <c r="H90" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+        <v>5.75</v>
+      </c>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>low-mid $28 x 38% less 10% condition, 3 source(s), high confidence — over budget cap</t>
+          <t>low-mid $28 x 38% less 10% condition, 3 source(s), high confidence</t>
         </is>
       </c>
     </row>
@@ -4824,10 +4824,10 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>10.12</v>
+        <v>10</v>
       </c>
       <c r="H91" t="n">
-        <v>11.64</v>
+        <v>11.5</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -4872,10 +4872,10 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>18.56</v>
+        <v>15</v>
       </c>
       <c r="H92" t="n">
-        <v>21.34</v>
+        <v>17.25</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -4920,10 +4920,10 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>20.25</v>
+        <v>20</v>
       </c>
       <c r="H93" t="n">
-        <v>23.29</v>
+        <v>23</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -4968,10 +4968,10 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>20.25</v>
+        <v>20</v>
       </c>
       <c r="H94" t="n">
-        <v>23.29</v>
+        <v>23</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -5016,10 +5016,10 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>25.31</v>
+        <v>25</v>
       </c>
       <c r="H95" t="n">
-        <v>29.11</v>
+        <v>28.75</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -5064,10 +5064,10 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>25.31</v>
+        <v>25</v>
       </c>
       <c r="H96" t="n">
-        <v>29.11</v>
+        <v>28.75</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>

</xml_diff>